<commit_message>
Update folder and add new pictures
</commit_message>
<xml_diff>
--- a/cost estimation sheet.xlsx
+++ b/cost estimation sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\Function hall_Cost estimation sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0FDE434-46CF-447B-9D70-B586A5D6CE30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28402EA8-2FA7-4953-BBF7-AAB4CA5F4CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D2A1664D-BF18-40D5-9F87-F85FB40B5178}"/>
   </bookViews>
@@ -881,6 +881,72 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -920,57 +986,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -978,21 +993,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1312,44 +1312,44 @@
   <dimension ref="A1:T50"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" customWidth="1"/>
+    <col min="1" max="1" width="11.88671875" customWidth="1"/>
     <col min="2" max="2" width="13.109375" customWidth="1"/>
     <col min="3" max="3" width="9.88671875" customWidth="1"/>
     <col min="4" max="4" width="14.77734375" customWidth="1"/>
     <col min="5" max="5" width="14.109375" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" customWidth="1"/>
     <col min="7" max="7" width="2.5546875" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" customWidth="1"/>
+    <col min="8" max="8" width="13.6640625" customWidth="1"/>
     <col min="9" max="9" width="16.109375" customWidth="1"/>
     <col min="11" max="11" width="9.6640625" customWidth="1"/>
     <col min="12" max="12" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="2.109375" customWidth="1"/>
     <col min="14" max="14" width="12.33203125" customWidth="1"/>
     <col min="15" max="15" width="11.33203125" customWidth="1"/>
-    <col min="16" max="16" width="11.44140625" customWidth="1"/>
-    <col min="17" max="17" width="10.109375" customWidth="1"/>
-    <col min="18" max="18" width="9.33203125" customWidth="1"/>
-    <col min="19" max="19" width="13" customWidth="1"/>
+    <col min="16" max="16" width="11.88671875" customWidth="1"/>
+    <col min="17" max="17" width="10.44140625" customWidth="1"/>
+    <col min="18" max="18" width="9.5546875" customWidth="1"/>
+    <col min="19" max="19" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
-      <c r="L1" s="52"/>
-      <c r="M1" s="52"/>
-      <c r="N1" s="52"/>
-      <c r="O1" s="53"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="49"/>
       <c r="P1" s="28" t="s">
         <v>47</v>
       </c>
@@ -1364,21 +1364,21 @@
       </c>
     </row>
     <row r="2" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="54"/>
-      <c r="B2" s="55"/>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="56"/>
+      <c r="A2" s="50"/>
+      <c r="B2" s="51"/>
+      <c r="C2" s="51"/>
+      <c r="D2" s="51"/>
+      <c r="E2" s="51"/>
+      <c r="F2" s="51"/>
+      <c r="G2" s="51"/>
+      <c r="H2" s="51"/>
+      <c r="I2" s="51"/>
+      <c r="J2" s="51"/>
+      <c r="K2" s="51"/>
+      <c r="L2" s="51"/>
+      <c r="M2" s="51"/>
+      <c r="N2" s="51"/>
+      <c r="O2" s="52"/>
       <c r="P2" s="11"/>
       <c r="Q2" s="29">
         <v>15</v>
@@ -1391,25 +1391,25 @@
       </c>
     </row>
     <row r="3" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="57"/>
-      <c r="B3" s="58"/>
-      <c r="C3" s="58"/>
-      <c r="D3" s="58"/>
-      <c r="E3" s="58"/>
-      <c r="F3" s="58"/>
-      <c r="G3" s="58"/>
-      <c r="H3" s="58"/>
-      <c r="I3" s="58"/>
-      <c r="J3" s="58"/>
-      <c r="K3" s="58"/>
-      <c r="L3" s="58"/>
-      <c r="M3" s="58"/>
-      <c r="N3" s="58"/>
-      <c r="O3" s="58"/>
-      <c r="P3" s="58"/>
-      <c r="Q3" s="58"/>
-      <c r="R3" s="58"/>
-      <c r="S3" s="59"/>
+      <c r="A3" s="53"/>
+      <c r="B3" s="54"/>
+      <c r="C3" s="54"/>
+      <c r="D3" s="54"/>
+      <c r="E3" s="54"/>
+      <c r="F3" s="54"/>
+      <c r="G3" s="54"/>
+      <c r="H3" s="54"/>
+      <c r="I3" s="54"/>
+      <c r="J3" s="54"/>
+      <c r="K3" s="54"/>
+      <c r="L3" s="54"/>
+      <c r="M3" s="54"/>
+      <c r="N3" s="54"/>
+      <c r="O3" s="54"/>
+      <c r="P3" s="54"/>
+      <c r="Q3" s="54"/>
+      <c r="R3" s="54"/>
+      <c r="S3" s="55"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -1434,23 +1434,23 @@
       <c r="H4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="63" t="s">
+      <c r="I4" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="J4" s="63"/>
-      <c r="K4" s="63" t="s">
+      <c r="J4" s="39"/>
+      <c r="K4" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="63"/>
+      <c r="L4" s="39"/>
       <c r="M4" s="5"/>
       <c r="N4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="O4" s="63" t="s">
+      <c r="O4" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="P4" s="63"/>
-      <c r="Q4" s="63"/>
+      <c r="P4" s="39"/>
+      <c r="Q4" s="39"/>
       <c r="R4" s="6"/>
       <c r="S4" s="7" t="s">
         <v>53</v>
@@ -1652,22 +1652,22 @@
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
-      <c r="H10" s="64" t="s">
+      <c r="H10" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="I10" s="64"/>
-      <c r="J10" s="64"/>
-      <c r="K10" s="64"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="38"/>
       <c r="L10" s="13">
         <f>SUM(L6:L8)</f>
         <v>1810050</v>
       </c>
       <c r="M10" s="14"/>
-      <c r="N10" s="64" t="s">
+      <c r="N10" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="O10" s="64"/>
-      <c r="P10" s="64"/>
+      <c r="O10" s="38"/>
+      <c r="P10" s="38"/>
       <c r="Q10" s="13">
         <f>Q6+Q7</f>
         <v>15000</v>
@@ -1679,25 +1679,25 @@
       </c>
     </row>
     <row r="11" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="71"/>
-      <c r="B11" s="72"/>
-      <c r="C11" s="72"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="72"/>
-      <c r="F11" s="72"/>
-      <c r="G11" s="72"/>
-      <c r="H11" s="72"/>
-      <c r="I11" s="72"/>
-      <c r="J11" s="72"/>
-      <c r="K11" s="72"/>
-      <c r="L11" s="72"/>
-      <c r="M11" s="72"/>
-      <c r="N11" s="72"/>
-      <c r="O11" s="72"/>
-      <c r="P11" s="72"/>
-      <c r="Q11" s="72"/>
-      <c r="R11" s="72"/>
-      <c r="S11" s="73"/>
+      <c r="A11" s="44"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
+      <c r="D11" s="45"/>
+      <c r="E11" s="45"/>
+      <c r="F11" s="45"/>
+      <c r="G11" s="45"/>
+      <c r="H11" s="45"/>
+      <c r="I11" s="45"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="45"/>
+      <c r="O11" s="45"/>
+      <c r="P11" s="45"/>
+      <c r="Q11" s="45"/>
+      <c r="R11" s="45"/>
+      <c r="S11" s="46"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -1722,23 +1722,23 @@
       <c r="H12" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I12" s="63" t="s">
+      <c r="I12" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="J12" s="63"/>
-      <c r="K12" s="63" t="s">
+      <c r="J12" s="39"/>
+      <c r="K12" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="L12" s="63"/>
+      <c r="L12" s="39"/>
       <c r="M12" s="5"/>
       <c r="N12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="O12" s="63" t="s">
+      <c r="O12" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="P12" s="63"/>
-      <c r="Q12" s="63"/>
+      <c r="P12" s="39"/>
+      <c r="Q12" s="39"/>
       <c r="R12" s="6"/>
       <c r="S12" s="18"/>
     </row>
@@ -1908,12 +1908,12 @@
       <c r="S15" s="9"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A16" s="61" t="s">
+      <c r="A16" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="62"/>
-      <c r="C16" s="62"/>
-      <c r="D16" s="62"/>
+      <c r="B16" s="41"/>
+      <c r="C16" s="41"/>
+      <c r="D16" s="41"/>
       <c r="E16" s="2">
         <f>SUM(E13:E15)</f>
         <v>10</v>
@@ -1944,22 +1944,22 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
-      <c r="H17" s="64" t="s">
+      <c r="H17" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="I17" s="64"/>
-      <c r="J17" s="64"/>
-      <c r="K17" s="64"/>
+      <c r="I17" s="38"/>
+      <c r="J17" s="38"/>
+      <c r="K17" s="38"/>
       <c r="L17" s="13">
         <f>SUM(L14:L15)</f>
         <v>25750</v>
       </c>
       <c r="M17" s="20"/>
-      <c r="N17" s="64" t="s">
+      <c r="N17" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="O17" s="64"/>
-      <c r="P17" s="64"/>
+      <c r="O17" s="38"/>
+      <c r="P17" s="38"/>
       <c r="Q17" s="13">
         <f>Q14+Q15</f>
         <v>15000</v>
@@ -1971,25 +1971,25 @@
       </c>
     </row>
     <row r="18" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="71"/>
-      <c r="B18" s="72"/>
-      <c r="C18" s="72"/>
-      <c r="D18" s="72"/>
-      <c r="E18" s="72"/>
-      <c r="F18" s="72"/>
-      <c r="G18" s="72"/>
-      <c r="H18" s="72"/>
-      <c r="I18" s="72"/>
-      <c r="J18" s="72"/>
-      <c r="K18" s="72"/>
-      <c r="L18" s="72"/>
-      <c r="M18" s="72"/>
-      <c r="N18" s="72"/>
-      <c r="O18" s="72"/>
-      <c r="P18" s="72"/>
-      <c r="Q18" s="72"/>
-      <c r="R18" s="72"/>
-      <c r="S18" s="73"/>
+      <c r="A18" s="44"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="45"/>
+      <c r="D18" s="45"/>
+      <c r="E18" s="45"/>
+      <c r="F18" s="45"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="45"/>
+      <c r="J18" s="45"/>
+      <c r="K18" s="45"/>
+      <c r="L18" s="45"/>
+      <c r="M18" s="45"/>
+      <c r="N18" s="45"/>
+      <c r="O18" s="45"/>
+      <c r="P18" s="45"/>
+      <c r="Q18" s="45"/>
+      <c r="R18" s="45"/>
+      <c r="S18" s="46"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
@@ -2012,23 +2012,23 @@
       <c r="H19" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I19" s="63" t="s">
+      <c r="I19" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="J19" s="63"/>
-      <c r="K19" s="63" t="s">
+      <c r="J19" s="39"/>
+      <c r="K19" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="L19" s="63"/>
+      <c r="L19" s="39"/>
       <c r="M19" s="5"/>
       <c r="N19" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="O19" s="63" t="s">
+      <c r="O19" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="P19" s="63"/>
-      <c r="Q19" s="63"/>
+      <c r="P19" s="39"/>
+      <c r="Q19" s="39"/>
       <c r="R19" s="6"/>
       <c r="S19" s="18"/>
     </row>
@@ -2231,22 +2231,22 @@
       <c r="E25" s="12"/>
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
-      <c r="H25" s="64" t="s">
+      <c r="H25" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="64"/>
-      <c r="J25" s="64"/>
-      <c r="K25" s="64"/>
+      <c r="I25" s="38"/>
+      <c r="J25" s="38"/>
+      <c r="K25" s="38"/>
       <c r="L25" s="13">
         <f>SUM(L21:L22)</f>
         <v>2850</v>
       </c>
       <c r="M25" s="14"/>
-      <c r="N25" s="64" t="s">
+      <c r="N25" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="O25" s="64"/>
-      <c r="P25" s="64"/>
+      <c r="O25" s="38"/>
+      <c r="P25" s="38"/>
       <c r="Q25" s="13">
         <f>Q21+Q22</f>
         <v>10200</v>
@@ -2258,25 +2258,25 @@
       </c>
     </row>
     <row r="26" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="71"/>
-      <c r="B26" s="72"/>
-      <c r="C26" s="72"/>
-      <c r="D26" s="72"/>
-      <c r="E26" s="72"/>
-      <c r="F26" s="72"/>
-      <c r="G26" s="72"/>
-      <c r="H26" s="72"/>
-      <c r="I26" s="72"/>
-      <c r="J26" s="72"/>
-      <c r="K26" s="72"/>
-      <c r="L26" s="72"/>
-      <c r="M26" s="72"/>
-      <c r="N26" s="72"/>
-      <c r="O26" s="72"/>
-      <c r="P26" s="72"/>
-      <c r="Q26" s="72"/>
-      <c r="R26" s="72"/>
-      <c r="S26" s="73"/>
+      <c r="A26" s="44"/>
+      <c r="B26" s="45"/>
+      <c r="C26" s="45"/>
+      <c r="D26" s="45"/>
+      <c r="E26" s="45"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="45"/>
+      <c r="H26" s="45"/>
+      <c r="I26" s="45"/>
+      <c r="J26" s="45"/>
+      <c r="K26" s="45"/>
+      <c r="L26" s="45"/>
+      <c r="M26" s="45"/>
+      <c r="N26" s="45"/>
+      <c r="O26" s="45"/>
+      <c r="P26" s="45"/>
+      <c r="Q26" s="45"/>
+      <c r="R26" s="45"/>
+      <c r="S26" s="46"/>
     </row>
     <row r="27" spans="1:19" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
@@ -2299,23 +2299,23 @@
       <c r="H27" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I27" s="63" t="s">
+      <c r="I27" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="J27" s="63"/>
-      <c r="K27" s="63" t="s">
+      <c r="J27" s="39"/>
+      <c r="K27" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="L27" s="63"/>
+      <c r="L27" s="39"/>
       <c r="M27" s="5"/>
       <c r="N27" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="O27" s="63" t="s">
+      <c r="O27" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="P27" s="63"/>
-      <c r="Q27" s="63"/>
+      <c r="P27" s="39"/>
+      <c r="Q27" s="39"/>
       <c r="R27" s="6"/>
       <c r="S27" s="18"/>
     </row>
@@ -2481,11 +2481,11 @@
       <c r="S30" s="9"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A31" s="61" t="s">
+      <c r="A31" s="40" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="62"/>
-      <c r="C31" s="62"/>
+      <c r="B31" s="41"/>
+      <c r="C31" s="41"/>
       <c r="D31" s="2">
         <f>SUM(D28:D30)</f>
         <v>550</v>
@@ -2522,9 +2522,9 @@
       <c r="S31" s="9"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A32" s="61"/>
-      <c r="B32" s="62"/>
-      <c r="C32" s="62"/>
+      <c r="A32" s="40"/>
+      <c r="B32" s="41"/>
+      <c r="C32" s="41"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
@@ -2550,22 +2550,22 @@
       <c r="E33" s="12"/>
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
-      <c r="H33" s="64" t="s">
+      <c r="H33" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="I33" s="64"/>
-      <c r="J33" s="64"/>
-      <c r="K33" s="64"/>
+      <c r="I33" s="38"/>
+      <c r="J33" s="38"/>
+      <c r="K33" s="38"/>
       <c r="L33" s="13">
         <f>L29+L30+L31</f>
         <v>71295</v>
       </c>
       <c r="M33" s="14"/>
-      <c r="N33" s="64" t="s">
+      <c r="N33" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="O33" s="64"/>
-      <c r="P33" s="64"/>
+      <c r="O33" s="38"/>
+      <c r="P33" s="38"/>
       <c r="Q33" s="13">
         <f>Q29+Q30</f>
         <v>13600</v>
@@ -2577,25 +2577,25 @@
       </c>
     </row>
     <row r="34" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="71"/>
-      <c r="B34" s="72"/>
-      <c r="C34" s="72"/>
-      <c r="D34" s="72"/>
-      <c r="E34" s="72"/>
-      <c r="F34" s="72"/>
-      <c r="G34" s="72"/>
-      <c r="H34" s="72"/>
-      <c r="I34" s="72"/>
-      <c r="J34" s="72"/>
-      <c r="K34" s="72"/>
-      <c r="L34" s="72"/>
-      <c r="M34" s="72"/>
-      <c r="N34" s="72"/>
-      <c r="O34" s="72"/>
-      <c r="P34" s="72"/>
-      <c r="Q34" s="72"/>
-      <c r="R34" s="72"/>
-      <c r="S34" s="73"/>
+      <c r="A34" s="44"/>
+      <c r="B34" s="45"/>
+      <c r="C34" s="45"/>
+      <c r="D34" s="45"/>
+      <c r="E34" s="45"/>
+      <c r="F34" s="45"/>
+      <c r="G34" s="45"/>
+      <c r="H34" s="45"/>
+      <c r="I34" s="45"/>
+      <c r="J34" s="45"/>
+      <c r="K34" s="45"/>
+      <c r="L34" s="45"/>
+      <c r="M34" s="45"/>
+      <c r="N34" s="45"/>
+      <c r="O34" s="45"/>
+      <c r="P34" s="45"/>
+      <c r="Q34" s="45"/>
+      <c r="R34" s="45"/>
+      <c r="S34" s="46"/>
     </row>
     <row r="35" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
@@ -2616,21 +2616,21 @@
       <c r="H35" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I35" s="63" t="s">
+      <c r="I35" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="J35" s="63"/>
-      <c r="K35" s="63" t="s">
+      <c r="J35" s="39"/>
+      <c r="K35" s="39" t="s">
         <v>11</v>
       </c>
-      <c r="L35" s="63"/>
+      <c r="L35" s="39"/>
       <c r="M35" s="5"/>
       <c r="N35" s="17"/>
-      <c r="O35" s="63" t="s">
+      <c r="O35" s="39" t="s">
         <v>41</v>
       </c>
-      <c r="P35" s="63"/>
-      <c r="Q35" s="63"/>
+      <c r="P35" s="39"/>
+      <c r="Q35" s="39"/>
       <c r="R35" s="6"/>
       <c r="S35" s="18"/>
     </row>
@@ -2830,22 +2830,22 @@
       <c r="E41" s="12"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
-      <c r="H41" s="65" t="s">
+      <c r="H41" s="57" t="s">
         <v>51</v>
       </c>
-      <c r="I41" s="66"/>
-      <c r="J41" s="66"/>
-      <c r="K41" s="67"/>
+      <c r="I41" s="58"/>
+      <c r="J41" s="58"/>
+      <c r="K41" s="59"/>
       <c r="L41" s="13">
         <f>L37+L38+L39</f>
         <v>91000</v>
       </c>
       <c r="M41" s="14"/>
-      <c r="N41" s="65" t="s">
+      <c r="N41" s="57" t="s">
         <v>54</v>
       </c>
-      <c r="O41" s="66"/>
-      <c r="P41" s="67"/>
+      <c r="O41" s="58"/>
+      <c r="P41" s="59"/>
       <c r="Q41" s="13">
         <f>Q37</f>
         <v>600000</v>
@@ -2857,25 +2857,25 @@
       </c>
     </row>
     <row r="42" spans="1:20" s="26" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="38"/>
-      <c r="B42" s="39"/>
-      <c r="C42" s="39"/>
-      <c r="D42" s="39"/>
-      <c r="E42" s="39"/>
-      <c r="F42" s="39"/>
-      <c r="G42" s="39"/>
-      <c r="H42" s="39"/>
-      <c r="I42" s="39"/>
-      <c r="J42" s="39"/>
-      <c r="K42" s="39"/>
-      <c r="L42" s="39"/>
-      <c r="M42" s="39"/>
-      <c r="N42" s="39"/>
-      <c r="O42" s="39"/>
-      <c r="P42" s="39"/>
-      <c r="Q42" s="39"/>
-      <c r="R42" s="39"/>
-      <c r="S42" s="40"/>
+      <c r="A42" s="60"/>
+      <c r="B42" s="61"/>
+      <c r="C42" s="61"/>
+      <c r="D42" s="61"/>
+      <c r="E42" s="61"/>
+      <c r="F42" s="61"/>
+      <c r="G42" s="61"/>
+      <c r="H42" s="61"/>
+      <c r="I42" s="61"/>
+      <c r="J42" s="61"/>
+      <c r="K42" s="61"/>
+      <c r="L42" s="61"/>
+      <c r="M42" s="61"/>
+      <c r="N42" s="61"/>
+      <c r="O42" s="61"/>
+      <c r="P42" s="61"/>
+      <c r="Q42" s="61"/>
+      <c r="R42" s="61"/>
+      <c r="S42" s="62"/>
       <c r="T42" s="37"/>
     </row>
     <row r="43" spans="1:20" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.35">
@@ -2886,20 +2886,20 @@
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
-      <c r="H43" s="41" t="s">
+      <c r="H43" s="63" t="s">
         <v>42</v>
       </c>
-      <c r="I43" s="42"/>
-      <c r="J43" s="42"/>
-      <c r="K43" s="42"/>
-      <c r="L43" s="43"/>
+      <c r="I43" s="64"/>
+      <c r="J43" s="64"/>
+      <c r="K43" s="64"/>
+      <c r="L43" s="65"/>
       <c r="M43" s="17"/>
-      <c r="N43" s="41" t="s">
+      <c r="N43" s="63" t="s">
         <v>43</v>
       </c>
-      <c r="O43" s="42"/>
-      <c r="P43" s="42"/>
-      <c r="Q43" s="43"/>
+      <c r="O43" s="64"/>
+      <c r="P43" s="64"/>
+      <c r="Q43" s="65"/>
       <c r="R43" s="34" t="s">
         <v>5</v>
       </c>
@@ -2917,22 +2917,22 @@
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
-      <c r="H44" s="48">
+      <c r="H44" s="70">
         <f>L41+L33+L25+L17+L10</f>
         <v>2000945</v>
       </c>
-      <c r="I44" s="49"/>
-      <c r="J44" s="49"/>
-      <c r="K44" s="49"/>
-      <c r="L44" s="50"/>
+      <c r="I44" s="71"/>
+      <c r="J44" s="71"/>
+      <c r="K44" s="71"/>
+      <c r="L44" s="72"/>
       <c r="M44" s="2"/>
-      <c r="N44" s="68">
+      <c r="N44" s="73">
         <f>Q41+Q33+Q25+Q10+Q17</f>
         <v>653800</v>
       </c>
-      <c r="O44" s="69"/>
-      <c r="P44" s="69"/>
-      <c r="Q44" s="70"/>
+      <c r="O44" s="74"/>
+      <c r="P44" s="74"/>
+      <c r="Q44" s="75"/>
       <c r="R44" s="1" t="s">
         <v>46</v>
       </c>
@@ -2958,10 +2958,10 @@
       <c r="N45" s="12"/>
       <c r="O45" s="12"/>
       <c r="P45" s="12"/>
-      <c r="Q45" s="74" t="s">
+      <c r="Q45" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="R45" s="75"/>
+      <c r="R45" s="43"/>
       <c r="S45" s="27">
         <f>S41*0.1</f>
         <v>69100</v>
@@ -3007,10 +3007,10 @@
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
       <c r="Q47" s="22"/>
-      <c r="R47" s="44" t="s">
+      <c r="R47" s="66" t="s">
         <v>50</v>
       </c>
-      <c r="S47" s="45"/>
+      <c r="S47" s="67"/>
     </row>
     <row r="48" spans="1:20" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2"/>
@@ -3030,27 +3030,43 @@
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
       <c r="Q48" s="22"/>
-      <c r="R48" s="46">
+      <c r="R48" s="68">
         <f>S10+S17+S25+S33+S41+S44+S45</f>
         <v>2856582.25</v>
       </c>
-      <c r="S48" s="47"/>
+      <c r="S48" s="69"/>
     </row>
     <row r="49" spans="15:16" x14ac:dyDescent="0.3">
-      <c r="O49" s="60"/>
-      <c r="P49" s="60"/>
+      <c r="O49" s="56"/>
+      <c r="P49" s="56"/>
     </row>
     <row r="50" spans="15:16" x14ac:dyDescent="0.3">
-      <c r="O50" s="60"/>
-      <c r="P50" s="60"/>
+      <c r="O50" s="56"/>
+      <c r="P50" s="56"/>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="N33:P33"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="Q45:R45"/>
+    <mergeCell ref="R47:S47"/>
+    <mergeCell ref="R48:S48"/>
+    <mergeCell ref="H44:L44"/>
+    <mergeCell ref="H43:L43"/>
+    <mergeCell ref="N44:Q44"/>
+    <mergeCell ref="A1:O2"/>
+    <mergeCell ref="A3:S3"/>
+    <mergeCell ref="O49:P49"/>
+    <mergeCell ref="O50:P50"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="H41:K41"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="H33:K33"/>
+    <mergeCell ref="I27:J27"/>
+    <mergeCell ref="N41:P41"/>
     <mergeCell ref="O4:Q4"/>
     <mergeCell ref="N10:P10"/>
     <mergeCell ref="O12:Q12"/>
@@ -3067,29 +3083,13 @@
     <mergeCell ref="A34:S34"/>
     <mergeCell ref="O35:Q35"/>
     <mergeCell ref="O19:Q19"/>
-    <mergeCell ref="A1:O2"/>
-    <mergeCell ref="A3:S3"/>
-    <mergeCell ref="O49:P49"/>
-    <mergeCell ref="O50:P50"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="H41:K41"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="H33:K33"/>
-    <mergeCell ref="I27:J27"/>
-    <mergeCell ref="N41:P41"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="O27:Q27"/>
+    <mergeCell ref="N33:P33"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="Q45:R45"/>
     <mergeCell ref="A42:S42"/>
     <mergeCell ref="N43:Q43"/>
-    <mergeCell ref="R47:S47"/>
-    <mergeCell ref="R48:S48"/>
-    <mergeCell ref="H44:L44"/>
-    <mergeCell ref="H43:L43"/>
-    <mergeCell ref="N44:Q44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update cost estimation sheet
</commit_message>
<xml_diff>
--- a/cost estimation sheet.xlsx
+++ b/cost estimation sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\Function hall_Cost estimation sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28402EA8-2FA7-4953-BBF7-AAB4CA5F4CAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEF33EE7-B204-40A7-8D04-DF80AC7D3708}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D2A1664D-BF18-40D5-9F87-F85FB40B5178}"/>
   </bookViews>
@@ -881,16 +881,103 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -899,54 +986,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -954,45 +993,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1317,9 +1317,9 @@
     <col min="3" max="3" width="9.88671875" customWidth="1"/>
     <col min="4" max="4" width="14.77734375" customWidth="1"/>
     <col min="5" max="5" width="14.109375" customWidth="1"/>
-    <col min="6" max="6" width="12.88671875" customWidth="1"/>
+    <col min="6" max="6" width="13.44140625" customWidth="1"/>
     <col min="7" max="7" width="2.5546875" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" customWidth="1"/>
+    <col min="8" max="8" width="13.33203125" customWidth="1"/>
     <col min="9" max="9" width="16.109375" customWidth="1"/>
     <col min="11" max="11" width="9.6640625" customWidth="1"/>
     <col min="12" max="12" width="10.5546875" bestFit="1" customWidth="1"/>
@@ -1328,28 +1328,28 @@
     <col min="15" max="15" width="11.33203125" customWidth="1"/>
     <col min="16" max="16" width="11.88671875" customWidth="1"/>
     <col min="17" max="17" width="10.44140625" customWidth="1"/>
-    <col min="18" max="18" width="9.5546875" customWidth="1"/>
+    <col min="18" max="18" width="9.6640625" customWidth="1"/>
     <col min="19" max="19" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="51" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="49"/>
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
+      <c r="K1" s="52"/>
+      <c r="L1" s="52"/>
+      <c r="M1" s="52"/>
+      <c r="N1" s="52"/>
+      <c r="O1" s="53"/>
       <c r="P1" s="28" t="s">
         <v>47</v>
       </c>
@@ -1364,21 +1364,21 @@
       </c>
     </row>
     <row r="2" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="50"/>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="H2" s="51"/>
-      <c r="I2" s="51"/>
-      <c r="J2" s="51"/>
-      <c r="K2" s="51"/>
-      <c r="L2" s="51"/>
-      <c r="M2" s="51"/>
-      <c r="N2" s="51"/>
-      <c r="O2" s="52"/>
+      <c r="A2" s="54"/>
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
+      <c r="O2" s="56"/>
       <c r="P2" s="11"/>
       <c r="Q2" s="29">
         <v>15</v>
@@ -1391,25 +1391,25 @@
       </c>
     </row>
     <row r="3" spans="1:19" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="53"/>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="54"/>
-      <c r="L3" s="54"/>
-      <c r="M3" s="54"/>
-      <c r="N3" s="54"/>
-      <c r="O3" s="54"/>
-      <c r="P3" s="54"/>
-      <c r="Q3" s="54"/>
-      <c r="R3" s="54"/>
-      <c r="S3" s="55"/>
+      <c r="A3" s="57"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="58"/>
+      <c r="J3" s="58"/>
+      <c r="K3" s="58"/>
+      <c r="L3" s="58"/>
+      <c r="M3" s="58"/>
+      <c r="N3" s="58"/>
+      <c r="O3" s="58"/>
+      <c r="P3" s="58"/>
+      <c r="Q3" s="58"/>
+      <c r="R3" s="58"/>
+      <c r="S3" s="59"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -1434,23 +1434,23 @@
       <c r="H4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="39" t="s">
+      <c r="I4" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39" t="s">
+      <c r="J4" s="63"/>
+      <c r="K4" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="39"/>
+      <c r="L4" s="63"/>
       <c r="M4" s="5"/>
       <c r="N4" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="O4" s="39" t="s">
+      <c r="O4" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="P4" s="39"/>
-      <c r="Q4" s="39"/>
+      <c r="P4" s="63"/>
+      <c r="Q4" s="63"/>
       <c r="R4" s="6"/>
       <c r="S4" s="7" t="s">
         <v>53</v>
@@ -1652,22 +1652,22 @@
       <c r="E10" s="12"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
-      <c r="H10" s="38" t="s">
+      <c r="H10" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="I10" s="38"/>
-      <c r="J10" s="38"/>
-      <c r="K10" s="38"/>
+      <c r="I10" s="64"/>
+      <c r="J10" s="64"/>
+      <c r="K10" s="64"/>
       <c r="L10" s="13">
         <f>SUM(L6:L8)</f>
         <v>1810050</v>
       </c>
       <c r="M10" s="14"/>
-      <c r="N10" s="38" t="s">
+      <c r="N10" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="O10" s="38"/>
-      <c r="P10" s="38"/>
+      <c r="O10" s="64"/>
+      <c r="P10" s="64"/>
       <c r="Q10" s="13">
         <f>Q6+Q7</f>
         <v>15000</v>
@@ -1679,25 +1679,25 @@
       </c>
     </row>
     <row r="11" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="44"/>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
-      <c r="D11" s="45"/>
-      <c r="E11" s="45"/>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="45"/>
-      <c r="I11" s="45"/>
-      <c r="J11" s="45"/>
-      <c r="K11" s="45"/>
-      <c r="L11" s="45"/>
-      <c r="M11" s="45"/>
-      <c r="N11" s="45"/>
-      <c r="O11" s="45"/>
-      <c r="P11" s="45"/>
-      <c r="Q11" s="45"/>
-      <c r="R11" s="45"/>
-      <c r="S11" s="46"/>
+      <c r="A11" s="68"/>
+      <c r="B11" s="69"/>
+      <c r="C11" s="69"/>
+      <c r="D11" s="69"/>
+      <c r="E11" s="69"/>
+      <c r="F11" s="69"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="69"/>
+      <c r="I11" s="69"/>
+      <c r="J11" s="69"/>
+      <c r="K11" s="69"/>
+      <c r="L11" s="69"/>
+      <c r="M11" s="69"/>
+      <c r="N11" s="69"/>
+      <c r="O11" s="69"/>
+      <c r="P11" s="69"/>
+      <c r="Q11" s="69"/>
+      <c r="R11" s="69"/>
+      <c r="S11" s="70"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
@@ -1722,23 +1722,23 @@
       <c r="H12" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I12" s="39" t="s">
+      <c r="I12" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="J12" s="39"/>
-      <c r="K12" s="39" t="s">
+      <c r="J12" s="63"/>
+      <c r="K12" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="L12" s="39"/>
+      <c r="L12" s="63"/>
       <c r="M12" s="5"/>
       <c r="N12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="O12" s="39" t="s">
+      <c r="O12" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="P12" s="39"/>
-      <c r="Q12" s="39"/>
+      <c r="P12" s="63"/>
+      <c r="Q12" s="63"/>
       <c r="R12" s="6"/>
       <c r="S12" s="18"/>
     </row>
@@ -1908,12 +1908,12 @@
       <c r="S15" s="9"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A16" s="40" t="s">
+      <c r="A16" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="41"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="41"/>
+      <c r="B16" s="62"/>
+      <c r="C16" s="62"/>
+      <c r="D16" s="62"/>
       <c r="E16" s="2">
         <f>SUM(E13:E15)</f>
         <v>10</v>
@@ -1944,22 +1944,22 @@
       <c r="E17" s="12"/>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
-      <c r="H17" s="38" t="s">
+      <c r="H17" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="I17" s="38"/>
-      <c r="J17" s="38"/>
-      <c r="K17" s="38"/>
+      <c r="I17" s="64"/>
+      <c r="J17" s="64"/>
+      <c r="K17" s="64"/>
       <c r="L17" s="13">
         <f>SUM(L14:L15)</f>
         <v>25750</v>
       </c>
       <c r="M17" s="20"/>
-      <c r="N17" s="38" t="s">
+      <c r="N17" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="O17" s="38"/>
-      <c r="P17" s="38"/>
+      <c r="O17" s="64"/>
+      <c r="P17" s="64"/>
       <c r="Q17" s="13">
         <f>Q14+Q15</f>
         <v>15000</v>
@@ -1971,25 +1971,25 @@
       </c>
     </row>
     <row r="18" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="44"/>
-      <c r="B18" s="45"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="45"/>
-      <c r="H18" s="45"/>
-      <c r="I18" s="45"/>
-      <c r="J18" s="45"/>
-      <c r="K18" s="45"/>
-      <c r="L18" s="45"/>
-      <c r="M18" s="45"/>
-      <c r="N18" s="45"/>
-      <c r="O18" s="45"/>
-      <c r="P18" s="45"/>
-      <c r="Q18" s="45"/>
-      <c r="R18" s="45"/>
-      <c r="S18" s="46"/>
+      <c r="A18" s="68"/>
+      <c r="B18" s="69"/>
+      <c r="C18" s="69"/>
+      <c r="D18" s="69"/>
+      <c r="E18" s="69"/>
+      <c r="F18" s="69"/>
+      <c r="G18" s="69"/>
+      <c r="H18" s="69"/>
+      <c r="I18" s="69"/>
+      <c r="J18" s="69"/>
+      <c r="K18" s="69"/>
+      <c r="L18" s="69"/>
+      <c r="M18" s="69"/>
+      <c r="N18" s="69"/>
+      <c r="O18" s="69"/>
+      <c r="P18" s="69"/>
+      <c r="Q18" s="69"/>
+      <c r="R18" s="69"/>
+      <c r="S18" s="70"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
@@ -2012,23 +2012,23 @@
       <c r="H19" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I19" s="39" t="s">
+      <c r="I19" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="J19" s="39"/>
-      <c r="K19" s="39" t="s">
+      <c r="J19" s="63"/>
+      <c r="K19" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="L19" s="39"/>
+      <c r="L19" s="63"/>
       <c r="M19" s="5"/>
       <c r="N19" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="O19" s="39" t="s">
+      <c r="O19" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="P19" s="39"/>
-      <c r="Q19" s="39"/>
+      <c r="P19" s="63"/>
+      <c r="Q19" s="63"/>
       <c r="R19" s="6"/>
       <c r="S19" s="18"/>
     </row>
@@ -2231,22 +2231,22 @@
       <c r="E25" s="12"/>
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
-      <c r="H25" s="38" t="s">
+      <c r="H25" s="64" t="s">
         <v>12</v>
       </c>
-      <c r="I25" s="38"/>
-      <c r="J25" s="38"/>
-      <c r="K25" s="38"/>
+      <c r="I25" s="64"/>
+      <c r="J25" s="64"/>
+      <c r="K25" s="64"/>
       <c r="L25" s="13">
         <f>SUM(L21:L22)</f>
         <v>2850</v>
       </c>
       <c r="M25" s="14"/>
-      <c r="N25" s="38" t="s">
+      <c r="N25" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="O25" s="38"/>
-      <c r="P25" s="38"/>
+      <c r="O25" s="64"/>
+      <c r="P25" s="64"/>
       <c r="Q25" s="13">
         <f>Q21+Q22</f>
         <v>10200</v>
@@ -2258,25 +2258,25 @@
       </c>
     </row>
     <row r="26" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="44"/>
-      <c r="B26" s="45"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
-      <c r="H26" s="45"/>
-      <c r="I26" s="45"/>
-      <c r="J26" s="45"/>
-      <c r="K26" s="45"/>
-      <c r="L26" s="45"/>
-      <c r="M26" s="45"/>
-      <c r="N26" s="45"/>
-      <c r="O26" s="45"/>
-      <c r="P26" s="45"/>
-      <c r="Q26" s="45"/>
-      <c r="R26" s="45"/>
-      <c r="S26" s="46"/>
+      <c r="A26" s="68"/>
+      <c r="B26" s="69"/>
+      <c r="C26" s="69"/>
+      <c r="D26" s="69"/>
+      <c r="E26" s="69"/>
+      <c r="F26" s="69"/>
+      <c r="G26" s="69"/>
+      <c r="H26" s="69"/>
+      <c r="I26" s="69"/>
+      <c r="J26" s="69"/>
+      <c r="K26" s="69"/>
+      <c r="L26" s="69"/>
+      <c r="M26" s="69"/>
+      <c r="N26" s="69"/>
+      <c r="O26" s="69"/>
+      <c r="P26" s="69"/>
+      <c r="Q26" s="69"/>
+      <c r="R26" s="69"/>
+      <c r="S26" s="70"/>
     </row>
     <row r="27" spans="1:19" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
@@ -2299,23 +2299,23 @@
       <c r="H27" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I27" s="39" t="s">
+      <c r="I27" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="J27" s="39"/>
-      <c r="K27" s="39" t="s">
+      <c r="J27" s="63"/>
+      <c r="K27" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="L27" s="39"/>
+      <c r="L27" s="63"/>
       <c r="M27" s="5"/>
       <c r="N27" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="O27" s="39" t="s">
+      <c r="O27" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="P27" s="39"/>
-      <c r="Q27" s="39"/>
+      <c r="P27" s="63"/>
+      <c r="Q27" s="63"/>
       <c r="R27" s="6"/>
       <c r="S27" s="18"/>
     </row>
@@ -2481,11 +2481,11 @@
       <c r="S30" s="9"/>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A31" s="40" t="s">
+      <c r="A31" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="B31" s="41"/>
-      <c r="C31" s="41"/>
+      <c r="B31" s="62"/>
+      <c r="C31" s="62"/>
       <c r="D31" s="2">
         <f>SUM(D28:D30)</f>
         <v>550</v>
@@ -2522,9 +2522,9 @@
       <c r="S31" s="9"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A32" s="40"/>
-      <c r="B32" s="41"/>
-      <c r="C32" s="41"/>
+      <c r="A32" s="61"/>
+      <c r="B32" s="62"/>
+      <c r="C32" s="62"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
@@ -2550,22 +2550,22 @@
       <c r="E33" s="12"/>
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
-      <c r="H33" s="38" t="s">
+      <c r="H33" s="64" t="s">
         <v>51</v>
       </c>
-      <c r="I33" s="38"/>
-      <c r="J33" s="38"/>
-      <c r="K33" s="38"/>
+      <c r="I33" s="64"/>
+      <c r="J33" s="64"/>
+      <c r="K33" s="64"/>
       <c r="L33" s="13">
         <f>L29+L30+L31</f>
         <v>71295</v>
       </c>
       <c r="M33" s="14"/>
-      <c r="N33" s="38" t="s">
+      <c r="N33" s="64" t="s">
         <v>52</v>
       </c>
-      <c r="O33" s="38"/>
-      <c r="P33" s="38"/>
+      <c r="O33" s="64"/>
+      <c r="P33" s="64"/>
       <c r="Q33" s="13">
         <f>Q29+Q30</f>
         <v>13600</v>
@@ -2577,25 +2577,25 @@
       </c>
     </row>
     <row r="34" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="44"/>
-      <c r="B34" s="45"/>
-      <c r="C34" s="45"/>
-      <c r="D34" s="45"/>
-      <c r="E34" s="45"/>
-      <c r="F34" s="45"/>
-      <c r="G34" s="45"/>
-      <c r="H34" s="45"/>
-      <c r="I34" s="45"/>
-      <c r="J34" s="45"/>
-      <c r="K34" s="45"/>
-      <c r="L34" s="45"/>
-      <c r="M34" s="45"/>
-      <c r="N34" s="45"/>
-      <c r="O34" s="45"/>
-      <c r="P34" s="45"/>
-      <c r="Q34" s="45"/>
-      <c r="R34" s="45"/>
-      <c r="S34" s="46"/>
+      <c r="A34" s="68"/>
+      <c r="B34" s="69"/>
+      <c r="C34" s="69"/>
+      <c r="D34" s="69"/>
+      <c r="E34" s="69"/>
+      <c r="F34" s="69"/>
+      <c r="G34" s="69"/>
+      <c r="H34" s="69"/>
+      <c r="I34" s="69"/>
+      <c r="J34" s="69"/>
+      <c r="K34" s="69"/>
+      <c r="L34" s="69"/>
+      <c r="M34" s="69"/>
+      <c r="N34" s="69"/>
+      <c r="O34" s="69"/>
+      <c r="P34" s="69"/>
+      <c r="Q34" s="69"/>
+      <c r="R34" s="69"/>
+      <c r="S34" s="70"/>
     </row>
     <row r="35" spans="1:20" ht="16.2" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
@@ -2616,21 +2616,21 @@
       <c r="H35" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="I35" s="39" t="s">
+      <c r="I35" s="63" t="s">
         <v>19</v>
       </c>
-      <c r="J35" s="39"/>
-      <c r="K35" s="39" t="s">
+      <c r="J35" s="63"/>
+      <c r="K35" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="L35" s="39"/>
+      <c r="L35" s="63"/>
       <c r="M35" s="5"/>
       <c r="N35" s="17"/>
-      <c r="O35" s="39" t="s">
+      <c r="O35" s="63" t="s">
         <v>41</v>
       </c>
-      <c r="P35" s="39"/>
-      <c r="Q35" s="39"/>
+      <c r="P35" s="63"/>
+      <c r="Q35" s="63"/>
       <c r="R35" s="6"/>
       <c r="S35" s="18"/>
     </row>
@@ -2830,22 +2830,22 @@
       <c r="E41" s="12"/>
       <c r="F41" s="12"/>
       <c r="G41" s="12"/>
-      <c r="H41" s="57" t="s">
+      <c r="H41" s="65" t="s">
         <v>51</v>
       </c>
-      <c r="I41" s="58"/>
-      <c r="J41" s="58"/>
-      <c r="K41" s="59"/>
+      <c r="I41" s="66"/>
+      <c r="J41" s="66"/>
+      <c r="K41" s="67"/>
       <c r="L41" s="13">
         <f>L37+L38+L39</f>
         <v>91000</v>
       </c>
       <c r="M41" s="14"/>
-      <c r="N41" s="57" t="s">
+      <c r="N41" s="65" t="s">
         <v>54</v>
       </c>
-      <c r="O41" s="58"/>
-      <c r="P41" s="59"/>
+      <c r="O41" s="66"/>
+      <c r="P41" s="67"/>
       <c r="Q41" s="13">
         <f>Q37</f>
         <v>600000</v>
@@ -2857,25 +2857,25 @@
       </c>
     </row>
     <row r="42" spans="1:20" s="26" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="60"/>
-      <c r="B42" s="61"/>
-      <c r="C42" s="61"/>
-      <c r="D42" s="61"/>
-      <c r="E42" s="61"/>
-      <c r="F42" s="61"/>
-      <c r="G42" s="61"/>
-      <c r="H42" s="61"/>
-      <c r="I42" s="61"/>
-      <c r="J42" s="61"/>
-      <c r="K42" s="61"/>
-      <c r="L42" s="61"/>
-      <c r="M42" s="61"/>
-      <c r="N42" s="61"/>
-      <c r="O42" s="61"/>
-      <c r="P42" s="61"/>
-      <c r="Q42" s="61"/>
-      <c r="R42" s="61"/>
-      <c r="S42" s="62"/>
+      <c r="A42" s="73"/>
+      <c r="B42" s="74"/>
+      <c r="C42" s="74"/>
+      <c r="D42" s="74"/>
+      <c r="E42" s="74"/>
+      <c r="F42" s="74"/>
+      <c r="G42" s="74"/>
+      <c r="H42" s="74"/>
+      <c r="I42" s="74"/>
+      <c r="J42" s="74"/>
+      <c r="K42" s="74"/>
+      <c r="L42" s="74"/>
+      <c r="M42" s="74"/>
+      <c r="N42" s="74"/>
+      <c r="O42" s="74"/>
+      <c r="P42" s="74"/>
+      <c r="Q42" s="74"/>
+      <c r="R42" s="74"/>
+      <c r="S42" s="75"/>
       <c r="T42" s="37"/>
     </row>
     <row r="43" spans="1:20" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.35">
@@ -2886,20 +2886,20 @@
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
       <c r="G43" s="6"/>
-      <c r="H43" s="63" t="s">
+      <c r="H43" s="45" t="s">
         <v>42</v>
       </c>
-      <c r="I43" s="64"/>
-      <c r="J43" s="64"/>
-      <c r="K43" s="64"/>
-      <c r="L43" s="65"/>
+      <c r="I43" s="46"/>
+      <c r="J43" s="46"/>
+      <c r="K43" s="46"/>
+      <c r="L43" s="47"/>
       <c r="M43" s="17"/>
-      <c r="N43" s="63" t="s">
+      <c r="N43" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="O43" s="64"/>
-      <c r="P43" s="64"/>
-      <c r="Q43" s="65"/>
+      <c r="O43" s="46"/>
+      <c r="P43" s="46"/>
+      <c r="Q43" s="47"/>
       <c r="R43" s="34" t="s">
         <v>5</v>
       </c>
@@ -2917,22 +2917,22 @@
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
-      <c r="H44" s="70">
+      <c r="H44" s="42">
         <f>L41+L33+L25+L17+L10</f>
         <v>2000945</v>
       </c>
-      <c r="I44" s="71"/>
-      <c r="J44" s="71"/>
-      <c r="K44" s="71"/>
-      <c r="L44" s="72"/>
+      <c r="I44" s="43"/>
+      <c r="J44" s="43"/>
+      <c r="K44" s="43"/>
+      <c r="L44" s="44"/>
       <c r="M44" s="2"/>
-      <c r="N44" s="73">
+      <c r="N44" s="48">
         <f>Q41+Q33+Q25+Q10+Q17</f>
         <v>653800</v>
       </c>
-      <c r="O44" s="74"/>
-      <c r="P44" s="74"/>
-      <c r="Q44" s="75"/>
+      <c r="O44" s="49"/>
+      <c r="P44" s="49"/>
+      <c r="Q44" s="50"/>
       <c r="R44" s="1" t="s">
         <v>46</v>
       </c>
@@ -2958,10 +2958,10 @@
       <c r="N45" s="12"/>
       <c r="O45" s="12"/>
       <c r="P45" s="12"/>
-      <c r="Q45" s="42" t="s">
+      <c r="Q45" s="71" t="s">
         <v>55</v>
       </c>
-      <c r="R45" s="43"/>
+      <c r="R45" s="72"/>
       <c r="S45" s="27">
         <f>S41*0.1</f>
         <v>69100</v>
@@ -3007,10 +3007,10 @@
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
       <c r="Q47" s="22"/>
-      <c r="R47" s="66" t="s">
+      <c r="R47" s="38" t="s">
         <v>50</v>
       </c>
-      <c r="S47" s="67"/>
+      <c r="S47" s="39"/>
     </row>
     <row r="48" spans="1:20" ht="19.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2"/>
@@ -3030,27 +3030,45 @@
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
       <c r="Q48" s="22"/>
-      <c r="R48" s="68">
+      <c r="R48" s="40">
         <f>S10+S17+S25+S33+S41+S44+S45</f>
         <v>2856582.25</v>
       </c>
-      <c r="S48" s="69"/>
+      <c r="S48" s="41"/>
     </row>
     <row r="49" spans="15:16" x14ac:dyDescent="0.3">
-      <c r="O49" s="56"/>
-      <c r="P49" s="56"/>
+      <c r="O49" s="60"/>
+      <c r="P49" s="60"/>
     </row>
     <row r="50" spans="15:16" x14ac:dyDescent="0.3">
-      <c r="O50" s="56"/>
-      <c r="P50" s="56"/>
+      <c r="O50" s="60"/>
+      <c r="P50" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="44">
-    <mergeCell ref="R47:S47"/>
-    <mergeCell ref="R48:S48"/>
-    <mergeCell ref="H44:L44"/>
-    <mergeCell ref="H43:L43"/>
-    <mergeCell ref="N44:Q44"/>
+    <mergeCell ref="N25:P25"/>
+    <mergeCell ref="O27:Q27"/>
+    <mergeCell ref="N33:P33"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="Q45:R45"/>
+    <mergeCell ref="A42:S42"/>
+    <mergeCell ref="N43:Q43"/>
+    <mergeCell ref="O4:Q4"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="O12:Q12"/>
+    <mergeCell ref="N17:P17"/>
+    <mergeCell ref="I35:J35"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="K12:L12"/>
+    <mergeCell ref="A11:S11"/>
+    <mergeCell ref="A18:S18"/>
+    <mergeCell ref="A26:S26"/>
+    <mergeCell ref="A34:S34"/>
+    <mergeCell ref="O35:Q35"/>
+    <mergeCell ref="O19:Q19"/>
     <mergeCell ref="A1:O2"/>
     <mergeCell ref="A3:S3"/>
     <mergeCell ref="O49:P49"/>
@@ -3067,29 +3085,11 @@
     <mergeCell ref="H33:K33"/>
     <mergeCell ref="I27:J27"/>
     <mergeCell ref="N41:P41"/>
-    <mergeCell ref="O4:Q4"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="O12:Q12"/>
-    <mergeCell ref="N17:P17"/>
-    <mergeCell ref="I35:J35"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="A11:S11"/>
-    <mergeCell ref="A18:S18"/>
-    <mergeCell ref="A26:S26"/>
-    <mergeCell ref="A34:S34"/>
-    <mergeCell ref="O35:Q35"/>
-    <mergeCell ref="O19:Q19"/>
-    <mergeCell ref="N25:P25"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="N33:P33"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="Q45:R45"/>
-    <mergeCell ref="A42:S42"/>
-    <mergeCell ref="N43:Q43"/>
+    <mergeCell ref="R47:S47"/>
+    <mergeCell ref="R48:S48"/>
+    <mergeCell ref="H44:L44"/>
+    <mergeCell ref="H43:L43"/>
+    <mergeCell ref="N44:Q44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>